<commit_message>
fix: recapture clean Hanoi preview
</commit_message>
<xml_diff>
--- a/Hanoi/hanoi.xlsx
+++ b/Hanoi/hanoi.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318F0F06-F621-D54C-8A9A-A53D90EEB373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F052688-BECD-A649-8227-86481E9F6919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15840" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -2057,20 +2057,20 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4622,28 +4622,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1">
-      <c r="A1" s="132" t="s">
+      <c r="A1" s="134" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="132"/>
-      <c r="C1" s="132"/>
-      <c r="D1" s="132"/>
-      <c r="E1" s="132"/>
-      <c r="F1" s="132"/>
-      <c r="G1" s="132"/>
-      <c r="H1" s="132"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
+      <c r="D1" s="134"/>
+      <c r="E1" s="134"/>
+      <c r="F1" s="134"/>
+      <c r="G1" s="134"/>
+      <c r="H1" s="134"/>
     </row>
     <row r="2" spans="1:8" ht="26" customHeight="1">
-      <c r="A2" s="133" t="s">
+      <c r="A2" s="135" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="133"/>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
+      <c r="B2" s="135"/>
+      <c r="C2" s="135"/>
+      <c r="D2" s="135"/>
+      <c r="E2" s="135"/>
+      <c r="F2" s="135"/>
+      <c r="G2" s="135"/>
+      <c r="H2" s="135"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1">
       <c r="A3" s="121"/>
@@ -4656,52 +4656,52 @@
       <c r="H3" s="121"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
-      <c r="A4" s="134" t="s">
+      <c r="A4" s="133" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="134"/>
-      <c r="C4" s="134"/>
-      <c r="D4" s="134"/>
-      <c r="E4" s="134"/>
-      <c r="F4" s="134"/>
-      <c r="G4" s="134"/>
-      <c r="H4" s="134"/>
+      <c r="B4" s="133"/>
+      <c r="C4" s="133"/>
+      <c r="D4" s="133"/>
+      <c r="E4" s="133"/>
+      <c r="F4" s="133"/>
+      <c r="G4" s="133"/>
+      <c r="H4" s="133"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
-      <c r="A5" s="131" t="s">
+      <c r="A5" s="132" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="131"/>
-      <c r="C5" s="131"/>
-      <c r="D5" s="131"/>
-      <c r="E5" s="131"/>
-      <c r="F5" s="131"/>
-      <c r="G5" s="131"/>
-      <c r="H5" s="131"/>
+      <c r="B5" s="132"/>
+      <c r="C5" s="132"/>
+      <c r="D5" s="132"/>
+      <c r="E5" s="132"/>
+      <c r="F5" s="132"/>
+      <c r="G5" s="132"/>
+      <c r="H5" s="132"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
-      <c r="A6" s="131" t="s">
+      <c r="A6" s="132" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="131"/>
-      <c r="C6" s="131"/>
-      <c r="D6" s="131"/>
-      <c r="E6" s="131"/>
-      <c r="F6" s="131"/>
-      <c r="G6" s="131"/>
-      <c r="H6" s="131"/>
+      <c r="B6" s="132"/>
+      <c r="C6" s="132"/>
+      <c r="D6" s="132"/>
+      <c r="E6" s="132"/>
+      <c r="F6" s="132"/>
+      <c r="G6" s="132"/>
+      <c r="H6" s="132"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="131" t="s">
+      <c r="A7" s="132" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="131"/>
-      <c r="C7" s="131"/>
-      <c r="D7" s="131"/>
-      <c r="E7" s="131"/>
-      <c r="F7" s="131"/>
-      <c r="G7" s="131"/>
-      <c r="H7" s="131"/>
+      <c r="B7" s="132"/>
+      <c r="C7" s="132"/>
+      <c r="D7" s="132"/>
+      <c r="E7" s="132"/>
+      <c r="F7" s="132"/>
+      <c r="G7" s="132"/>
+      <c r="H7" s="132"/>
     </row>
     <row r="8" spans="1:8" ht="10" customHeight="1">
       <c r="A8" s="121"/>
@@ -4714,28 +4714,28 @@
       <c r="H8" s="121"/>
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1">
-      <c r="A9" s="134" t="s">
+      <c r="A9" s="133" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="134"/>
-      <c r="C9" s="134"/>
-      <c r="D9" s="134"/>
-      <c r="E9" s="134"/>
-      <c r="F9" s="134"/>
-      <c r="G9" s="134"/>
-      <c r="H9" s="134"/>
+      <c r="B9" s="133"/>
+      <c r="C9" s="133"/>
+      <c r="D9" s="133"/>
+      <c r="E9" s="133"/>
+      <c r="F9" s="133"/>
+      <c r="G9" s="133"/>
+      <c r="H9" s="133"/>
     </row>
     <row r="10" spans="1:8" ht="40" customHeight="1">
-      <c r="A10" s="131" t="s">
+      <c r="A10" s="132" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="131"/>
-      <c r="C10" s="131"/>
-      <c r="D10" s="131"/>
-      <c r="E10" s="131"/>
-      <c r="F10" s="131"/>
-      <c r="G10" s="131"/>
-      <c r="H10" s="131"/>
+      <c r="B10" s="132"/>
+      <c r="C10" s="132"/>
+      <c r="D10" s="132"/>
+      <c r="E10" s="132"/>
+      <c r="F10" s="132"/>
+      <c r="G10" s="132"/>
+      <c r="H10" s="132"/>
     </row>
     <row r="11" spans="1:8" ht="10" customHeight="1">
       <c r="A11" s="121"/>
@@ -4748,52 +4748,52 @@
       <c r="H11" s="121"/>
     </row>
     <row r="12" spans="1:8" ht="24" customHeight="1">
-      <c r="A12" s="134" t="s">
+      <c r="A12" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="134"/>
-      <c r="C12" s="134"/>
-      <c r="D12" s="134"/>
-      <c r="E12" s="134"/>
-      <c r="F12" s="134"/>
-      <c r="G12" s="134"/>
-      <c r="H12" s="134"/>
+      <c r="B12" s="133"/>
+      <c r="C12" s="133"/>
+      <c r="D12" s="133"/>
+      <c r="E12" s="133"/>
+      <c r="F12" s="133"/>
+      <c r="G12" s="133"/>
+      <c r="H12" s="133"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="131" t="s">
+      <c r="A13" s="132" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="131"/>
-      <c r="C13" s="131"/>
-      <c r="D13" s="131"/>
-      <c r="E13" s="131"/>
-      <c r="F13" s="131"/>
-      <c r="G13" s="131"/>
-      <c r="H13" s="131"/>
+      <c r="B13" s="132"/>
+      <c r="C13" s="132"/>
+      <c r="D13" s="132"/>
+      <c r="E13" s="132"/>
+      <c r="F13" s="132"/>
+      <c r="G13" s="132"/>
+      <c r="H13" s="132"/>
     </row>
     <row r="14" spans="1:8" ht="24" customHeight="1">
-      <c r="A14" s="131" t="s">
+      <c r="A14" s="132" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="131"/>
-      <c r="C14" s="131"/>
-      <c r="D14" s="131"/>
-      <c r="E14" s="131"/>
-      <c r="F14" s="131"/>
-      <c r="G14" s="131"/>
-      <c r="H14" s="131"/>
+      <c r="B14" s="132"/>
+      <c r="C14" s="132"/>
+      <c r="D14" s="132"/>
+      <c r="E14" s="132"/>
+      <c r="F14" s="132"/>
+      <c r="G14" s="132"/>
+      <c r="H14" s="132"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1">
-      <c r="A15" s="131" t="s">
+      <c r="A15" s="132" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="131"/>
-      <c r="C15" s="131"/>
-      <c r="D15" s="131"/>
-      <c r="E15" s="131"/>
-      <c r="F15" s="131"/>
-      <c r="G15" s="131"/>
-      <c r="H15" s="131"/>
+      <c r="B15" s="132"/>
+      <c r="C15" s="132"/>
+      <c r="D15" s="132"/>
+      <c r="E15" s="132"/>
+      <c r="F15" s="132"/>
+      <c r="G15" s="132"/>
+      <c r="H15" s="132"/>
     </row>
     <row r="16" spans="1:8" ht="10" customHeight="1">
       <c r="A16" s="121"/>
@@ -4806,40 +4806,40 @@
       <c r="H16" s="121"/>
     </row>
     <row r="17" spans="1:8" ht="24" customHeight="1">
-      <c r="A17" s="134" t="s">
+      <c r="A17" s="133" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="134"/>
-      <c r="C17" s="134"/>
-      <c r="D17" s="134"/>
-      <c r="E17" s="134"/>
-      <c r="F17" s="134"/>
-      <c r="G17" s="134"/>
-      <c r="H17" s="134"/>
+      <c r="B17" s="133"/>
+      <c r="C17" s="133"/>
+      <c r="D17" s="133"/>
+      <c r="E17" s="133"/>
+      <c r="F17" s="133"/>
+      <c r="G17" s="133"/>
+      <c r="H17" s="133"/>
     </row>
     <row r="18" spans="1:8" ht="28" customHeight="1">
-      <c r="A18" s="131" t="s">
+      <c r="A18" s="132" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="131"/>
-      <c r="C18" s="131"/>
-      <c r="D18" s="131"/>
-      <c r="E18" s="131"/>
-      <c r="F18" s="131"/>
-      <c r="G18" s="131"/>
-      <c r="H18" s="131"/>
+      <c r="B18" s="132"/>
+      <c r="C18" s="132"/>
+      <c r="D18" s="132"/>
+      <c r="E18" s="132"/>
+      <c r="F18" s="132"/>
+      <c r="G18" s="132"/>
+      <c r="H18" s="132"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1">
-      <c r="A19" s="131" t="s">
+      <c r="A19" s="132" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="131"/>
-      <c r="C19" s="131"/>
-      <c r="D19" s="131"/>
-      <c r="E19" s="131"/>
-      <c r="F19" s="131"/>
-      <c r="G19" s="131"/>
-      <c r="H19" s="131"/>
+      <c r="B19" s="132"/>
+      <c r="C19" s="132"/>
+      <c r="D19" s="132"/>
+      <c r="E19" s="132"/>
+      <c r="F19" s="132"/>
+      <c r="G19" s="132"/>
+      <c r="H19" s="132"/>
     </row>
     <row r="20" spans="1:8" ht="10" customHeight="1">
       <c r="A20" s="121"/>
@@ -4852,64 +4852,64 @@
       <c r="H20" s="121"/>
     </row>
     <row r="21" spans="1:8" ht="24" customHeight="1">
-      <c r="A21" s="134" t="s">
+      <c r="A21" s="133" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="134"/>
-      <c r="C21" s="134"/>
-      <c r="D21" s="134"/>
-      <c r="E21" s="134"/>
-      <c r="F21" s="134"/>
-      <c r="G21" s="134"/>
-      <c r="H21" s="134"/>
+      <c r="B21" s="133"/>
+      <c r="C21" s="133"/>
+      <c r="D21" s="133"/>
+      <c r="E21" s="133"/>
+      <c r="F21" s="133"/>
+      <c r="G21" s="133"/>
+      <c r="H21" s="133"/>
     </row>
     <row r="22" spans="1:8" ht="26" customHeight="1">
-      <c r="A22" s="131" t="s">
+      <c r="A22" s="132" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="131"/>
-      <c r="C22" s="131"/>
-      <c r="D22" s="131"/>
-      <c r="E22" s="131"/>
-      <c r="F22" s="131"/>
-      <c r="G22" s="131"/>
-      <c r="H22" s="131"/>
+      <c r="B22" s="132"/>
+      <c r="C22" s="132"/>
+      <c r="D22" s="132"/>
+      <c r="E22" s="132"/>
+      <c r="F22" s="132"/>
+      <c r="G22" s="132"/>
+      <c r="H22" s="132"/>
     </row>
     <row r="23" spans="1:8" ht="28" customHeight="1">
-      <c r="A23" s="131" t="s">
+      <c r="A23" s="132" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="131"/>
-      <c r="C23" s="131"/>
-      <c r="D23" s="131"/>
-      <c r="E23" s="131"/>
-      <c r="F23" s="131"/>
-      <c r="G23" s="131"/>
-      <c r="H23" s="131"/>
+      <c r="B23" s="132"/>
+      <c r="C23" s="132"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="132"/>
+      <c r="F23" s="132"/>
+      <c r="G23" s="132"/>
+      <c r="H23" s="132"/>
     </row>
     <row r="24" spans="1:8" ht="26" customHeight="1">
-      <c r="A24" s="131" t="s">
+      <c r="A24" s="132" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="131"/>
-      <c r="C24" s="131"/>
-      <c r="D24" s="131"/>
-      <c r="E24" s="131"/>
-      <c r="F24" s="131"/>
-      <c r="G24" s="131"/>
-      <c r="H24" s="131"/>
+      <c r="B24" s="132"/>
+      <c r="C24" s="132"/>
+      <c r="D24" s="132"/>
+      <c r="E24" s="132"/>
+      <c r="F24" s="132"/>
+      <c r="G24" s="132"/>
+      <c r="H24" s="132"/>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1">
-      <c r="A25" s="131" t="s">
+      <c r="A25" s="132" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="131"/>
-      <c r="C25" s="131"/>
-      <c r="D25" s="131"/>
-      <c r="E25" s="131"/>
-      <c r="F25" s="131"/>
-      <c r="G25" s="131"/>
-      <c r="H25" s="131"/>
+      <c r="B25" s="132"/>
+      <c r="C25" s="132"/>
+      <c r="D25" s="132"/>
+      <c r="E25" s="132"/>
+      <c r="F25" s="132"/>
+      <c r="G25" s="132"/>
+      <c r="H25" s="132"/>
     </row>
     <row r="26" spans="1:8" ht="10" customHeight="1">
       <c r="A26" s="121"/>
@@ -4922,28 +4922,28 @@
       <c r="H26" s="121"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1">
-      <c r="A27" s="134" t="s">
+      <c r="A27" s="133" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="134"/>
-      <c r="C27" s="134"/>
-      <c r="D27" s="134"/>
-      <c r="E27" s="134"/>
-      <c r="F27" s="134"/>
-      <c r="G27" s="134"/>
-      <c r="H27" s="134"/>
+      <c r="B27" s="133"/>
+      <c r="C27" s="133"/>
+      <c r="D27" s="133"/>
+      <c r="E27" s="133"/>
+      <c r="F27" s="133"/>
+      <c r="G27" s="133"/>
+      <c r="H27" s="133"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
-      <c r="A28" s="131" t="s">
+      <c r="A28" s="132" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="131"/>
-      <c r="C28" s="131"/>
-      <c r="D28" s="131"/>
-      <c r="E28" s="131"/>
-      <c r="F28" s="131"/>
-      <c r="G28" s="131"/>
-      <c r="H28" s="131"/>
+      <c r="B28" s="132"/>
+      <c r="C28" s="132"/>
+      <c r="D28" s="132"/>
+      <c r="E28" s="132"/>
+      <c r="F28" s="132"/>
+      <c r="G28" s="132"/>
+      <c r="H28" s="132"/>
     </row>
     <row r="29" spans="1:8" ht="10" customHeight="1">
       <c r="A29" s="121"/>
@@ -4956,50 +4956,49 @@
       <c r="H29" s="121"/>
     </row>
     <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="134" t="s">
+      <c r="A30" s="133" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="134"/>
-      <c r="C30" s="134"/>
-      <c r="D30" s="134"/>
-      <c r="E30" s="134"/>
-      <c r="F30" s="134"/>
-      <c r="G30" s="134"/>
-      <c r="H30" s="134"/>
+      <c r="B30" s="133"/>
+      <c r="C30" s="133"/>
+      <c r="D30" s="133"/>
+      <c r="E30" s="133"/>
+      <c r="F30" s="133"/>
+      <c r="G30" s="133"/>
+      <c r="H30" s="133"/>
     </row>
     <row r="31" spans="1:8" ht="34" customHeight="1">
-      <c r="A31" s="131" t="s">
+      <c r="A31" s="132" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="131"/>
-      <c r="C31" s="131"/>
-      <c r="D31" s="131"/>
-      <c r="E31" s="131"/>
-      <c r="F31" s="131"/>
-      <c r="G31" s="131"/>
-      <c r="H31" s="131"/>
+      <c r="B31" s="132"/>
+      <c r="C31" s="132"/>
+      <c r="D31" s="132"/>
+      <c r="E31" s="132"/>
+      <c r="F31" s="132"/>
+      <c r="G31" s="132"/>
+      <c r="H31" s="132"/>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1">
-      <c r="A32" s="135" t="s">
+      <c r="A32" s="131" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="135"/>
-      <c r="C32" s="135"/>
-      <c r="D32" s="135"/>
-      <c r="E32" s="135"/>
-      <c r="F32" s="135"/>
-      <c r="G32" s="135"/>
-      <c r="H32" s="135"/>
+      <c r="B32" s="131"/>
+      <c r="C32" s="131"/>
+      <c r="D32" s="131"/>
+      <c r="E32" s="131"/>
+      <c r="F32" s="131"/>
+      <c r="G32" s="131"/>
+      <c r="H32" s="131"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A10:H10"/>
@@ -5012,12 +5011,13 @@
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: handle error-valued Hanoi inputs
</commit_message>
<xml_diff>
--- a/Hanoi/hanoi.xlsx
+++ b/Hanoi/hanoi.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F052688-BECD-A649-8227-86481E9F6919}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D65E59-4541-B341-A4BC-CBAA9233BBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="15840" xr2:uid="{82D447F9-66A8-4F40-88AB-946121063596}"/>
   </bookViews>
@@ -2057,20 +2057,20 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="97" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4089,7 +4089,7 @@
         <v>61</v>
       </c>
       <c r="B13" s="30" t="str" cm="1">
-        <f t="array" ref="B13">_xlfn.LET(_xlpm.d,HN_CLAMP_DISKS($B$5),_xlpm.s,HN_EFFECTIVE_STEP($B$6,HN_MAX_STEP(_xlpm.d)),IF(AND($B$5=_xlpm.d,$B$6=_xlpm.s),"Inputs valid","Display adjusted to "&amp;_xlpm.d&amp;" disks / step "&amp;_xlpm.s))</f>
+        <f t="array" ref="B13">_xlfn.LET(_xlpm.d,HN_CLAMP_DISKS($B$5),_xlpm.s,HN_EFFECTIVE_STEP($B$6,HN_MAX_STEP(_xlpm.d)),IF(IFERROR(AND($B$5=_xlpm.d,$B$6=_xlpm.s),FALSE),"Inputs valid","Display adjusted to "&amp;_xlpm.d&amp;" disks / step "&amp;_xlpm.s))</f>
         <v>Inputs valid</v>
       </c>
       <c r="C13" s="92"/>
@@ -4622,28 +4622,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="34" customHeight="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="132" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
-      <c r="D1" s="134"/>
-      <c r="E1" s="134"/>
-      <c r="F1" s="134"/>
-      <c r="G1" s="134"/>
-      <c r="H1" s="134"/>
+      <c r="B1" s="132"/>
+      <c r="C1" s="132"/>
+      <c r="D1" s="132"/>
+      <c r="E1" s="132"/>
+      <c r="F1" s="132"/>
+      <c r="G1" s="132"/>
+      <c r="H1" s="132"/>
     </row>
     <row r="2" spans="1:8" ht="26" customHeight="1">
-      <c r="A2" s="135" t="s">
+      <c r="A2" s="133" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-      <c r="D2" s="135"/>
-      <c r="E2" s="135"/>
-      <c r="F2" s="135"/>
-      <c r="G2" s="135"/>
-      <c r="H2" s="135"/>
+      <c r="B2" s="133"/>
+      <c r="C2" s="133"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
     </row>
     <row r="3" spans="1:8" ht="10" customHeight="1">
       <c r="A3" s="121"/>
@@ -4656,52 +4656,52 @@
       <c r="H3" s="121"/>
     </row>
     <row r="4" spans="1:8" ht="24" customHeight="1">
-      <c r="A4" s="133" t="s">
+      <c r="A4" s="134" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="133"/>
-      <c r="C4" s="133"/>
-      <c r="D4" s="133"/>
-      <c r="E4" s="133"/>
-      <c r="F4" s="133"/>
-      <c r="G4" s="133"/>
-      <c r="H4" s="133"/>
+      <c r="B4" s="134"/>
+      <c r="C4" s="134"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="134"/>
+      <c r="F4" s="134"/>
+      <c r="G4" s="134"/>
+      <c r="H4" s="134"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
-      <c r="A5" s="132" t="s">
+      <c r="A5" s="131" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="132"/>
-      <c r="C5" s="132"/>
-      <c r="D5" s="132"/>
-      <c r="E5" s="132"/>
-      <c r="F5" s="132"/>
-      <c r="G5" s="132"/>
-      <c r="H5" s="132"/>
+      <c r="B5" s="131"/>
+      <c r="C5" s="131"/>
+      <c r="D5" s="131"/>
+      <c r="E5" s="131"/>
+      <c r="F5" s="131"/>
+      <c r="G5" s="131"/>
+      <c r="H5" s="131"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
-      <c r="A6" s="132" t="s">
+      <c r="A6" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="132"/>
-      <c r="C6" s="132"/>
-      <c r="D6" s="132"/>
-      <c r="E6" s="132"/>
-      <c r="F6" s="132"/>
-      <c r="G6" s="132"/>
-      <c r="H6" s="132"/>
+      <c r="B6" s="131"/>
+      <c r="C6" s="131"/>
+      <c r="D6" s="131"/>
+      <c r="E6" s="131"/>
+      <c r="F6" s="131"/>
+      <c r="G6" s="131"/>
+      <c r="H6" s="131"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1">
-      <c r="A7" s="132" t="s">
+      <c r="A7" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="B7" s="132"/>
-      <c r="C7" s="132"/>
-      <c r="D7" s="132"/>
-      <c r="E7" s="132"/>
-      <c r="F7" s="132"/>
-      <c r="G7" s="132"/>
-      <c r="H7" s="132"/>
+      <c r="B7" s="131"/>
+      <c r="C7" s="131"/>
+      <c r="D7" s="131"/>
+      <c r="E7" s="131"/>
+      <c r="F7" s="131"/>
+      <c r="G7" s="131"/>
+      <c r="H7" s="131"/>
     </row>
     <row r="8" spans="1:8" ht="10" customHeight="1">
       <c r="A8" s="121"/>
@@ -4714,28 +4714,28 @@
       <c r="H8" s="121"/>
     </row>
     <row r="9" spans="1:8" ht="24" customHeight="1">
-      <c r="A9" s="133" t="s">
+      <c r="A9" s="134" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="133"/>
-      <c r="C9" s="133"/>
-      <c r="D9" s="133"/>
-      <c r="E9" s="133"/>
-      <c r="F9" s="133"/>
-      <c r="G9" s="133"/>
-      <c r="H9" s="133"/>
+      <c r="B9" s="134"/>
+      <c r="C9" s="134"/>
+      <c r="D9" s="134"/>
+      <c r="E9" s="134"/>
+      <c r="F9" s="134"/>
+      <c r="G9" s="134"/>
+      <c r="H9" s="134"/>
     </row>
     <row r="10" spans="1:8" ht="40" customHeight="1">
-      <c r="A10" s="132" t="s">
+      <c r="A10" s="131" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="132"/>
-      <c r="C10" s="132"/>
-      <c r="D10" s="132"/>
-      <c r="E10" s="132"/>
-      <c r="F10" s="132"/>
-      <c r="G10" s="132"/>
-      <c r="H10" s="132"/>
+      <c r="B10" s="131"/>
+      <c r="C10" s="131"/>
+      <c r="D10" s="131"/>
+      <c r="E10" s="131"/>
+      <c r="F10" s="131"/>
+      <c r="G10" s="131"/>
+      <c r="H10" s="131"/>
     </row>
     <row r="11" spans="1:8" ht="10" customHeight="1">
       <c r="A11" s="121"/>
@@ -4748,52 +4748,52 @@
       <c r="H11" s="121"/>
     </row>
     <row r="12" spans="1:8" ht="24" customHeight="1">
-      <c r="A12" s="133" t="s">
+      <c r="A12" s="134" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="133"/>
-      <c r="C12" s="133"/>
-      <c r="D12" s="133"/>
-      <c r="E12" s="133"/>
-      <c r="F12" s="133"/>
-      <c r="G12" s="133"/>
-      <c r="H12" s="133"/>
+      <c r="B12" s="134"/>
+      <c r="C12" s="134"/>
+      <c r="D12" s="134"/>
+      <c r="E12" s="134"/>
+      <c r="F12" s="134"/>
+      <c r="G12" s="134"/>
+      <c r="H12" s="134"/>
     </row>
     <row r="13" spans="1:8" ht="26" customHeight="1">
-      <c r="A13" s="132" t="s">
+      <c r="A13" s="131" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="132"/>
-      <c r="C13" s="132"/>
-      <c r="D13" s="132"/>
-      <c r="E13" s="132"/>
-      <c r="F13" s="132"/>
-      <c r="G13" s="132"/>
-      <c r="H13" s="132"/>
+      <c r="B13" s="131"/>
+      <c r="C13" s="131"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="131"/>
+      <c r="F13" s="131"/>
+      <c r="G13" s="131"/>
+      <c r="H13" s="131"/>
     </row>
     <row r="14" spans="1:8" ht="24" customHeight="1">
-      <c r="A14" s="132" t="s">
+      <c r="A14" s="131" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="132"/>
-      <c r="C14" s="132"/>
-      <c r="D14" s="132"/>
-      <c r="E14" s="132"/>
-      <c r="F14" s="132"/>
-      <c r="G14" s="132"/>
-      <c r="H14" s="132"/>
+      <c r="B14" s="131"/>
+      <c r="C14" s="131"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="131"/>
+      <c r="F14" s="131"/>
+      <c r="G14" s="131"/>
+      <c r="H14" s="131"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1">
-      <c r="A15" s="132" t="s">
+      <c r="A15" s="131" t="s">
         <v>47</v>
       </c>
-      <c r="B15" s="132"/>
-      <c r="C15" s="132"/>
-      <c r="D15" s="132"/>
-      <c r="E15" s="132"/>
-      <c r="F15" s="132"/>
-      <c r="G15" s="132"/>
-      <c r="H15" s="132"/>
+      <c r="B15" s="131"/>
+      <c r="C15" s="131"/>
+      <c r="D15" s="131"/>
+      <c r="E15" s="131"/>
+      <c r="F15" s="131"/>
+      <c r="G15" s="131"/>
+      <c r="H15" s="131"/>
     </row>
     <row r="16" spans="1:8" ht="10" customHeight="1">
       <c r="A16" s="121"/>
@@ -4806,40 +4806,40 @@
       <c r="H16" s="121"/>
     </row>
     <row r="17" spans="1:8" ht="24" customHeight="1">
-      <c r="A17" s="133" t="s">
+      <c r="A17" s="134" t="s">
         <v>48</v>
       </c>
-      <c r="B17" s="133"/>
-      <c r="C17" s="133"/>
-      <c r="D17" s="133"/>
-      <c r="E17" s="133"/>
-      <c r="F17" s="133"/>
-      <c r="G17" s="133"/>
-      <c r="H17" s="133"/>
+      <c r="B17" s="134"/>
+      <c r="C17" s="134"/>
+      <c r="D17" s="134"/>
+      <c r="E17" s="134"/>
+      <c r="F17" s="134"/>
+      <c r="G17" s="134"/>
+      <c r="H17" s="134"/>
     </row>
     <row r="18" spans="1:8" ht="28" customHeight="1">
-      <c r="A18" s="132" t="s">
+      <c r="A18" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="B18" s="132"/>
-      <c r="C18" s="132"/>
-      <c r="D18" s="132"/>
-      <c r="E18" s="132"/>
-      <c r="F18" s="132"/>
-      <c r="G18" s="132"/>
-      <c r="H18" s="132"/>
+      <c r="B18" s="131"/>
+      <c r="C18" s="131"/>
+      <c r="D18" s="131"/>
+      <c r="E18" s="131"/>
+      <c r="F18" s="131"/>
+      <c r="G18" s="131"/>
+      <c r="H18" s="131"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1">
-      <c r="A19" s="132" t="s">
+      <c r="A19" s="131" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="132"/>
-      <c r="C19" s="132"/>
-      <c r="D19" s="132"/>
-      <c r="E19" s="132"/>
-      <c r="F19" s="132"/>
-      <c r="G19" s="132"/>
-      <c r="H19" s="132"/>
+      <c r="B19" s="131"/>
+      <c r="C19" s="131"/>
+      <c r="D19" s="131"/>
+      <c r="E19" s="131"/>
+      <c r="F19" s="131"/>
+      <c r="G19" s="131"/>
+      <c r="H19" s="131"/>
     </row>
     <row r="20" spans="1:8" ht="10" customHeight="1">
       <c r="A20" s="121"/>
@@ -4852,64 +4852,64 @@
       <c r="H20" s="121"/>
     </row>
     <row r="21" spans="1:8" ht="24" customHeight="1">
-      <c r="A21" s="133" t="s">
+      <c r="A21" s="134" t="s">
         <v>51</v>
       </c>
-      <c r="B21" s="133"/>
-      <c r="C21" s="133"/>
-      <c r="D21" s="133"/>
-      <c r="E21" s="133"/>
-      <c r="F21" s="133"/>
-      <c r="G21" s="133"/>
-      <c r="H21" s="133"/>
+      <c r="B21" s="134"/>
+      <c r="C21" s="134"/>
+      <c r="D21" s="134"/>
+      <c r="E21" s="134"/>
+      <c r="F21" s="134"/>
+      <c r="G21" s="134"/>
+      <c r="H21" s="134"/>
     </row>
     <row r="22" spans="1:8" ht="26" customHeight="1">
-      <c r="A22" s="132" t="s">
+      <c r="A22" s="131" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="132"/>
-      <c r="C22" s="132"/>
-      <c r="D22" s="132"/>
-      <c r="E22" s="132"/>
-      <c r="F22" s="132"/>
-      <c r="G22" s="132"/>
-      <c r="H22" s="132"/>
+      <c r="B22" s="131"/>
+      <c r="C22" s="131"/>
+      <c r="D22" s="131"/>
+      <c r="E22" s="131"/>
+      <c r="F22" s="131"/>
+      <c r="G22" s="131"/>
+      <c r="H22" s="131"/>
     </row>
     <row r="23" spans="1:8" ht="28" customHeight="1">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="131" t="s">
         <v>53</v>
       </c>
-      <c r="B23" s="132"/>
-      <c r="C23" s="132"/>
-      <c r="D23" s="132"/>
-      <c r="E23" s="132"/>
-      <c r="F23" s="132"/>
-      <c r="G23" s="132"/>
-      <c r="H23" s="132"/>
+      <c r="B23" s="131"/>
+      <c r="C23" s="131"/>
+      <c r="D23" s="131"/>
+      <c r="E23" s="131"/>
+      <c r="F23" s="131"/>
+      <c r="G23" s="131"/>
+      <c r="H23" s="131"/>
     </row>
     <row r="24" spans="1:8" ht="26" customHeight="1">
-      <c r="A24" s="132" t="s">
+      <c r="A24" s="131" t="s">
         <v>54</v>
       </c>
-      <c r="B24" s="132"/>
-      <c r="C24" s="132"/>
-      <c r="D24" s="132"/>
-      <c r="E24" s="132"/>
-      <c r="F24" s="132"/>
-      <c r="G24" s="132"/>
-      <c r="H24" s="132"/>
+      <c r="B24" s="131"/>
+      <c r="C24" s="131"/>
+      <c r="D24" s="131"/>
+      <c r="E24" s="131"/>
+      <c r="F24" s="131"/>
+      <c r="G24" s="131"/>
+      <c r="H24" s="131"/>
     </row>
     <row r="25" spans="1:8" ht="36" customHeight="1">
-      <c r="A25" s="132" t="s">
+      <c r="A25" s="131" t="s">
         <v>55</v>
       </c>
-      <c r="B25" s="132"/>
-      <c r="C25" s="132"/>
-      <c r="D25" s="132"/>
-      <c r="E25" s="132"/>
-      <c r="F25" s="132"/>
-      <c r="G25" s="132"/>
-      <c r="H25" s="132"/>
+      <c r="B25" s="131"/>
+      <c r="C25" s="131"/>
+      <c r="D25" s="131"/>
+      <c r="E25" s="131"/>
+      <c r="F25" s="131"/>
+      <c r="G25" s="131"/>
+      <c r="H25" s="131"/>
     </row>
     <row r="26" spans="1:8" ht="10" customHeight="1">
       <c r="A26" s="121"/>
@@ -4922,28 +4922,28 @@
       <c r="H26" s="121"/>
     </row>
     <row r="27" spans="1:8" ht="24" customHeight="1">
-      <c r="A27" s="133" t="s">
+      <c r="A27" s="134" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="133"/>
-      <c r="C27" s="133"/>
-      <c r="D27" s="133"/>
-      <c r="E27" s="133"/>
-      <c r="F27" s="133"/>
-      <c r="G27" s="133"/>
-      <c r="H27" s="133"/>
+      <c r="B27" s="134"/>
+      <c r="C27" s="134"/>
+      <c r="D27" s="134"/>
+      <c r="E27" s="134"/>
+      <c r="F27" s="134"/>
+      <c r="G27" s="134"/>
+      <c r="H27" s="134"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1">
-      <c r="A28" s="132" t="s">
+      <c r="A28" s="131" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="132"/>
-      <c r="C28" s="132"/>
-      <c r="D28" s="132"/>
-      <c r="E28" s="132"/>
-      <c r="F28" s="132"/>
-      <c r="G28" s="132"/>
-      <c r="H28" s="132"/>
+      <c r="B28" s="131"/>
+      <c r="C28" s="131"/>
+      <c r="D28" s="131"/>
+      <c r="E28" s="131"/>
+      <c r="F28" s="131"/>
+      <c r="G28" s="131"/>
+      <c r="H28" s="131"/>
     </row>
     <row r="29" spans="1:8" ht="10" customHeight="1">
       <c r="A29" s="121"/>
@@ -4956,49 +4956,50 @@
       <c r="H29" s="121"/>
     </row>
     <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="133" t="s">
+      <c r="A30" s="134" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="133"/>
-      <c r="C30" s="133"/>
-      <c r="D30" s="133"/>
-      <c r="E30" s="133"/>
-      <c r="F30" s="133"/>
-      <c r="G30" s="133"/>
-      <c r="H30" s="133"/>
+      <c r="B30" s="134"/>
+      <c r="C30" s="134"/>
+      <c r="D30" s="134"/>
+      <c r="E30" s="134"/>
+      <c r="F30" s="134"/>
+      <c r="G30" s="134"/>
+      <c r="H30" s="134"/>
     </row>
     <row r="31" spans="1:8" ht="34" customHeight="1">
-      <c r="A31" s="132" t="s">
+      <c r="A31" s="131" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="132"/>
-      <c r="C31" s="132"/>
-      <c r="D31" s="132"/>
-      <c r="E31" s="132"/>
-      <c r="F31" s="132"/>
-      <c r="G31" s="132"/>
-      <c r="H31" s="132"/>
+      <c r="B31" s="131"/>
+      <c r="C31" s="131"/>
+      <c r="D31" s="131"/>
+      <c r="E31" s="131"/>
+      <c r="F31" s="131"/>
+      <c r="G31" s="131"/>
+      <c r="H31" s="131"/>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1">
-      <c r="A32" s="131" t="s">
+      <c r="A32" s="135" t="s">
         <v>60</v>
       </c>
-      <c r="B32" s="131"/>
-      <c r="C32" s="131"/>
-      <c r="D32" s="131"/>
-      <c r="E32" s="131"/>
-      <c r="F32" s="131"/>
-      <c r="G32" s="131"/>
-      <c r="H32" s="131"/>
+      <c r="B32" s="135"/>
+      <c r="C32" s="135"/>
+      <c r="D32" s="135"/>
+      <c r="E32" s="135"/>
+      <c r="F32" s="135"/>
+      <c r="G32" s="135"/>
+      <c r="H32" s="135"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A10:H10"/>
@@ -5011,13 +5012,12 @@
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="A21:H21"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A27:H27"/>
-    <mergeCell ref="A28:H28"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>